<commit_message>
Update multitrack GaN data + Update chosen devices' loss break down
</commit_message>
<xml_diff>
--- a/Switch Functions/SiC Data tf.xlsx
+++ b/Switch Functions/SiC Data tf.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Component\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA72262-FB58-4686-9934-CBBBCA88E774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B3697F-219D-45F5-94A3-2554D2D71A1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>Part Number</t>
   </si>
@@ -183,12 +183,6 @@
   </si>
   <si>
     <t>Q_gs</t>
-  </si>
-  <si>
-    <t>larger than t_f provided in the datasheet</t>
-  </si>
-  <si>
-    <t>t_f provided in the datasheet sincce not enough data is given to do the calculation</t>
   </si>
 </sst>
 </file>
@@ -300,7 +294,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -347,11 +341,17 @@
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -635,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.54296875" customWidth="1"/>
@@ -1156,7 +1156,7 @@
       <c r="W6" s="2">
         <v>7</v>
       </c>
-      <c r="X6" s="18">
+      <c r="X6" s="16">
         <v>3.8</v>
       </c>
       <c r="Y6" s="2">
@@ -1247,7 +1247,7 @@
       <c r="W7" s="2">
         <v>7</v>
       </c>
-      <c r="X7" s="18">
+      <c r="X7" s="16">
         <v>3.8</v>
       </c>
       <c r="Y7" s="2">
@@ -1338,7 +1338,7 @@
       <c r="W8" s="2">
         <v>7.2</v>
       </c>
-      <c r="X8" s="18">
+      <c r="X8" s="16">
         <v>3.8</v>
       </c>
       <c r="Y8" s="2">
@@ -1538,11 +1538,29 @@
       <c r="A11" s="4"/>
       <c r="B11" s="11"/>
     </row>
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="Q13" s="17"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="18"/>
+      <c r="T13" s="18"/>
+      <c r="U13" s="18"/>
+      <c r="V13" s="18"/>
+      <c r="W13" s="18"/>
+      <c r="X13" s="18"/>
+      <c r="Y13" s="17"/>
+      <c r="Z13" s="18"/>
+    </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="Q14" s="16"/>
-      <c r="R14" s="17" t="s">
-        <v>49</v>
-      </c>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="18"/>
+      <c r="T14" s="18"/>
+      <c r="U14" s="18"/>
+      <c r="V14" s="18"/>
+      <c r="W14" s="18"/>
+      <c r="X14" s="18"/>
+      <c r="Y14" s="17"/>
+      <c r="Z14" s="18"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15" s="4"/>
@@ -1561,10 +1579,28 @@
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" s="6"/>
-      <c r="Q15" s="14"/>
-      <c r="R15" s="17" t="s">
-        <v>50</v>
-      </c>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="19"/>
+      <c r="S15" s="18"/>
+      <c r="T15" s="18"/>
+      <c r="U15" s="18"/>
+      <c r="V15" s="18"/>
+      <c r="W15" s="18"/>
+      <c r="X15" s="18"/>
+      <c r="Y15" s="17"/>
+      <c r="Z15" s="18"/>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+      <c r="Q16" s="17"/>
+      <c r="R16" s="18"/>
+      <c r="S16" s="18"/>
+      <c r="T16" s="18"/>
+      <c r="U16" s="18"/>
+      <c r="V16" s="18"/>
+      <c r="W16" s="18"/>
+      <c r="X16" s="18"/>
+      <c r="Y16" s="17"/>
+      <c r="Z16" s="18"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q10">

</xml_diff>